<commit_message>
Add persistent weekly homework reports and escalation actions
</commit_message>
<xml_diff>
--- a/homework-app/templates/summary-t1.xlsx
+++ b/homework-app/templates/summary-t1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\17_Incomplete Homework\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kochu\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B030C795-74A4-4539-B9B9-5A8AD0D98F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D52BC9-F0EB-4825-953F-D431ADC91FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10815" yWindow="0" windowWidth="18030" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="wk6" sheetId="28" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="171">
   <si>
     <t>小一 (P1)</t>
   </si>
@@ -700,6 +700,18 @@
   </si>
   <si>
     <t>已留堂1次</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>已留堂2次</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>已留堂3次</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>已留堂4次</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -751,7 +763,7 @@
       <charset val="136"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -788,6 +800,30 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -821,7 +857,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -873,6 +909,12 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -880,6 +922,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1313,82 +1364,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
     </row>
     <row r="2" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
     </row>
     <row r="3" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="19" t="s">
         <v>166</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
     </row>
     <row r="4" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19" t="s">
+      <c r="C4" s="21"/>
+      <c r="D4" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19" t="s">
+      <c r="I4" s="21"/>
+      <c r="J4" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19" t="s">
+      <c r="K4" s="21"/>
+      <c r="L4" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="19"/>
+      <c r="M4" s="21"/>
     </row>
     <row r="5" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -1414,10 +1465,10 @@
       <c r="I5" s="4">
         <v>4</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="J5" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5" s="18">
         <v>4</v>
       </c>
       <c r="L5" s="3" t="s">
@@ -1576,6 +1627,9 @@
         <v>137</v>
       </c>
       <c r="M9" s="4"/>
+      <c r="N9" s="22" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="10" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -1611,6 +1665,9 @@
         <v>138</v>
       </c>
       <c r="M10" s="4"/>
+      <c r="N10" s="23" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="11" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
@@ -1644,6 +1701,9 @@
       </c>
       <c r="M11" s="8">
         <v>7</v>
+      </c>
+      <c r="N11" s="24" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -2445,82 +2505,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
     </row>
     <row r="2" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
     </row>
     <row r="3" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="19" t="s">
         <v>164</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
     </row>
     <row r="4" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19" t="s">
+      <c r="C4" s="21"/>
+      <c r="D4" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19" t="s">
+      <c r="I4" s="21"/>
+      <c r="J4" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19" t="s">
+      <c r="K4" s="21"/>
+      <c r="L4" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="19"/>
+      <c r="M4" s="21"/>
     </row>
     <row r="5" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -3549,82 +3609,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
     </row>
     <row r="2" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
     </row>
     <row r="3" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
     </row>
     <row r="4" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19" t="s">
+      <c r="C4" s="21"/>
+      <c r="D4" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19" t="s">
+      <c r="I4" s="21"/>
+      <c r="J4" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19" t="s">
+      <c r="K4" s="21"/>
+      <c r="L4" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="19"/>
+      <c r="M4" s="21"/>
     </row>
     <row r="5" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -4625,82 +4685,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
     </row>
     <row r="2" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
     </row>
     <row r="3" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
     </row>
     <row r="4" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19" t="s">
+      <c r="C4" s="21"/>
+      <c r="D4" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19" t="s">
+      <c r="I4" s="21"/>
+      <c r="J4" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19" t="s">
+      <c r="K4" s="21"/>
+      <c r="L4" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="19"/>
+      <c r="M4" s="21"/>
     </row>
     <row r="5" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -5637,82 +5697,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
     </row>
     <row r="2" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+      <c r="M2" s="20"/>
     </row>
     <row r="3" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="19" t="s">
         <v>159</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
     </row>
     <row r="4" spans="1:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19" t="s">
+      <c r="C4" s="21"/>
+      <c r="D4" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19" t="s">
+      <c r="I4" s="21"/>
+      <c r="J4" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19" t="s">
+      <c r="K4" s="21"/>
+      <c r="L4" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="19"/>
+      <c r="M4" s="21"/>
     </row>
     <row r="5" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">

</xml_diff>